<commit_message>
ONs: columna "Divisa de pago" con MEP/CCL (domicilio de pago de 1816)
La columna Divisa pasa de "USD" (poco informativo) a la divisa de pago real:
MEP o CCL, según el domicilio de pago del bono (campo domicilio_pago de las
condiciones de emisión de 1816: Argentina->MEP, Estados Unidos->CCL/cable).
Scrapeado por instrumento (private API); 44 MEP, 38 CCL. Columna renombrada a
"Divisa de pago". Los ⚡ auto-agregados muestran "—" hasta que se les scrapee el
domicilio en la revisión semanal (el API público no lo expone).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Instrumentos.xlsx
+++ b/Instrumentos.xlsx
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2873" uniqueCount="447">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2873" uniqueCount="449">
   <si>
     <t>Ticker</t>
   </si>
@@ -1393,6 +1393,12 @@
   <si>
     <t>B. Mariva 2027</t>
   </si>
+  <si>
+    <t>CCL</t>
+  </si>
+  <si>
+    <t>MEP</t>
+  </si>
 </sst>
 </file>
 
@@ -3899,21 +3905,21 @@
   <dimension ref="A1:E83"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="5" width="10" customWidth="1"/>
+    <col min="1" max="1" width="10"/>
+    <col min="2" max="2" width="26"/>
+    <col min="3" max="3" width="18"/>
+    <col min="4" max="5" width="10"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="2" t="s">
-        <v>169</v>
+        <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>170</v>
+        <v>108</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>171</v>
+        <v>3</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>172</v>
@@ -3936,7 +3942,7 @@
         <v>176</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -3953,7 +3959,7 @@
         <v>176</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -3970,7 +3976,7 @@
         <v>176</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -3987,7 +3993,7 @@
         <v>176</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -4004,7 +4010,7 @@
         <v>176</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -4021,12 +4027,12 @@
         <v>176</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="1" t="s">
-        <v>188</v>
+        <v>89</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>189</v>
@@ -4038,7 +4044,7 @@
         <v>176</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -4055,7 +4061,7 @@
         <v>176</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -4072,7 +4078,7 @@
         <v>176</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -4089,7 +4095,7 @@
         <v>176</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -4106,7 +4112,7 @@
         <v>176</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -4123,7 +4129,7 @@
         <v>176</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -4140,7 +4146,7 @@
         <v>176</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -4157,7 +4163,7 @@
         <v>176</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -4174,7 +4180,7 @@
         <v>176</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -4191,7 +4197,7 @@
         <v>176</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -4208,7 +4214,7 @@
         <v>176</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -4225,7 +4231,7 @@
         <v>176</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -4242,7 +4248,7 @@
         <v>176</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -4259,12 +4265,12 @@
         <v>176</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="1" t="s">
-        <v>216</v>
+        <v>88</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>217</v>
@@ -4276,7 +4282,7 @@
         <v>176</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -4293,7 +4299,7 @@
         <v>176</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -4310,7 +4316,7 @@
         <v>176</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -4327,7 +4333,7 @@
         <v>176</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -4344,7 +4350,7 @@
         <v>176</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -4361,7 +4367,7 @@
         <v>176</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -4378,7 +4384,7 @@
         <v>176</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -4395,7 +4401,7 @@
         <v>176</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -4412,7 +4418,7 @@
         <v>176</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -4429,7 +4435,7 @@
         <v>176</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -4446,7 +4452,7 @@
         <v>176</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -4463,7 +4469,7 @@
         <v>176</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -4480,7 +4486,7 @@
         <v>242</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -4497,7 +4503,7 @@
         <v>242</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -4514,7 +4520,7 @@
         <v>242</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -4531,7 +4537,7 @@
         <v>242</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -4548,7 +4554,7 @@
         <v>242</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -4565,7 +4571,7 @@
         <v>242</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -4582,7 +4588,7 @@
         <v>242</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="41" spans="1:5">
@@ -4599,7 +4605,7 @@
         <v>242</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -4616,7 +4622,7 @@
         <v>242</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="43" spans="1:5">
@@ -4633,7 +4639,7 @@
         <v>242</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -4650,7 +4656,7 @@
         <v>242</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -4667,7 +4673,7 @@
         <v>242</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -4684,7 +4690,7 @@
         <v>242</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -4701,7 +4707,7 @@
         <v>242</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -4718,7 +4724,7 @@
         <v>242</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="49" spans="1:5">
@@ -4735,7 +4741,7 @@
         <v>242</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="50" spans="1:5">
@@ -4752,7 +4758,7 @@
         <v>242</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="51" spans="1:5">
@@ -4769,7 +4775,7 @@
         <v>242</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -4786,7 +4792,7 @@
         <v>242</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -4803,7 +4809,7 @@
         <v>242</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -4820,7 +4826,7 @@
         <v>242</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -4837,7 +4843,7 @@
         <v>242</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="56" spans="1:5">
@@ -4854,7 +4860,7 @@
         <v>242</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="57" spans="1:5">
@@ -4871,7 +4877,7 @@
         <v>242</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -4888,7 +4894,7 @@
         <v>242</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -4905,7 +4911,7 @@
         <v>242</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="60" spans="1:5">
@@ -4922,7 +4928,7 @@
         <v>242</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="61" spans="1:5">
@@ -4939,12 +4945,12 @@
         <v>242</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="62" spans="1:5">
       <c r="A62" s="1" t="s">
-        <v>296</v>
+        <v>87</v>
       </c>
       <c r="B62" s="1" t="s">
         <v>297</v>
@@ -4956,7 +4962,7 @@
         <v>242</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="63" spans="1:5">
@@ -4973,7 +4979,7 @@
         <v>242</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -4990,7 +4996,7 @@
         <v>242</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -5007,7 +5013,7 @@
         <v>242</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -5024,7 +5030,7 @@
         <v>242</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -5041,7 +5047,7 @@
         <v>242</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="68" spans="1:5">
@@ -5058,7 +5064,7 @@
         <v>242</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="69" spans="1:5">
@@ -5075,7 +5081,7 @@
         <v>242</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="70" spans="1:5">
@@ -5092,12 +5098,12 @@
         <v>242</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>177</v>
+        <v>447</v>
       </c>
     </row>
     <row r="71" spans="1:5">
       <c r="A71" s="1" t="s">
-        <v>314</v>
+        <v>86</v>
       </c>
       <c r="B71" s="1" t="s">
         <v>315</v>
@@ -5109,7 +5115,7 @@
         <v>242</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="72" spans="1:5">
@@ -5126,7 +5132,7 @@
         <v>242</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="73" spans="1:5">
@@ -5143,7 +5149,7 @@
         <v>242</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="74" spans="1:5">
@@ -5160,7 +5166,7 @@
         <v>242</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -5177,7 +5183,7 @@
         <v>242</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="76" spans="1:5">
@@ -5194,7 +5200,7 @@
         <v>242</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="77" spans="1:5">
@@ -5211,7 +5217,7 @@
         <v>242</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="78" spans="1:5">
@@ -5228,7 +5234,7 @@
         <v>242</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="79" spans="1:5">
@@ -5245,7 +5251,7 @@
         <v>242</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="80" spans="1:5">
@@ -5262,7 +5268,7 @@
         <v>242</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="81" spans="1:5">
@@ -5279,7 +5285,7 @@
         <v>242</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="82" spans="1:5">
@@ -5296,7 +5302,7 @@
         <v>242</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
     <row r="83" spans="1:5">
@@ -5313,7 +5319,7 @@
         <v>242</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>177</v>
+        <v>448</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Instrumentos: agregar LECAP S16O6 y USD Linked D15E7
- S16O6 (LECAP): emisión 2026-07-31, venc 2026-10-16, TEM 2,05%.
- D15E7 (USD Linked): emisión 2026-07-31, venc 2027-01-15, TC inicial 1499,84, margen 0.
- Editado vía XML directo para preservar los valores cacheados de las
  fórmulas de las otras hojas (openpyxl los pierde y no hay LibreOffice
  para recalcular).
- Pendientes sin cargar (siguen en el detector): TMVE8 (dual nuevo tipo), LBS26 (subsoberano).
</commit_message>
<xml_diff>
--- a/Instrumentos.xlsx
+++ b/Instrumentos.xlsx
@@ -2138,13 +2138,33 @@
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>S16O6</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>LECAP</t>
+        </is>
+      </c>
+      <c r="C18" s="3">
+        <v>46234</v>
+      </c>
+      <c r="D18" s="3">
+        <v>46311</v>
+      </c>
+      <c r="E18" s="1">
+        <v>2.05</v>
+      </c>
+      <c r="F18" s="7">
+        <f>DAYS360(C18,D18)/30</f>
+        <v>2.533333333333333</v>
+      </c>
+      <c r="G18" s="1">
+        <f>100*(1+E18/100)^F18</f>
+        <v>105.2752519814636</v>
+      </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
@@ -37652,7 +37672,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35C12C03-5D2E-4402-9FEE-10F6AEE7B245}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="6" width="19.1640625" customWidth="1"/>
@@ -37835,6 +37855,30 @@
         <v>1474.74</v>
       </c>
       <c r="F10" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>D15E7</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>Linked</t>
+        </is>
+      </c>
+      <c r="C11" s="3">
+        <v>46234</v>
+      </c>
+      <c r="D11" s="3">
+        <v>46402</v>
+      </c>
+      <c r="E11" s="1">
+        <v>1499.84</v>
+      </c>
+      <c r="F11" s="1">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Sumar 3 ONs nuevas: VSCZD, MR44D y LQC1D
Detectadas en la revisión semanal: emitidas en los últimos 180 días y con más de
100.000 nominales de volumen promedio.

  VSCZD  Vista Energy 2029             ley local
  MR44D  GEMSA - CTR 2036              ley local
  LQC1D  PCR - Luz de Tres Picos 2034  ley NY

La divisa de pago queda vacía en las dos de ley local (muestran "—"): en el
universo actual ley local es 44 MEP contra 6 CCL, así que no se puede inferir;
sale del domicilio_pago al scrapear el cashflow. En LQC1D se pone CCL porque
ley NY es 32 de 32 en el universo.

La hoja se regeneró por cirugía de XML en vez de round-trip con openpyxl: el
libro tiene 1429 fórmulas en otras hojas y openpyxl les borra el valor cacheado,
que es lo que lee el frontend. Verificado post-escritura: 1429 fórmulas intactas,
13 hojas, y la única con distinto nº de filas es ONs (82 -> 85).

Quedan con ⚡ hasta que se scrapee el cronograma de flujos.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Instrumentos.xlsx
+++ b/Instrumentos.xlsx
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2873" uniqueCount="449">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2883" uniqueCount="455">
   <si>
     <t>Ticker</t>
   </si>
@@ -1399,6 +1399,24 @@
   <si>
     <t>MEP</t>
   </si>
+  <si>
+    <t>VSCZD</t>
+  </si>
+  <si>
+    <t>Vista Energy 2029</t>
+  </si>
+  <si>
+    <t>LQC1D</t>
+  </si>
+  <si>
+    <t>PCR - Luz de Tres Picos 2034</t>
+  </si>
+  <si>
+    <t>MR44D</t>
+  </si>
+  <si>
+    <t>GEMSA - CTR 2036</t>
+  </si>
 </sst>
 </file>
 
@@ -3922,7 +3940,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E83"/>
+  <dimension ref="A1:E86"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10"/>
@@ -3950,254 +3968,254 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="1" t="s">
-        <v>174</v>
+        <v>282</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>175</v>
+        <v>283</v>
       </c>
       <c r="C2" s="3">
-        <v>47036</v>
+        <v>46256</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="1" t="s">
-        <v>178</v>
+        <v>280</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>179</v>
+        <v>281</v>
       </c>
       <c r="C3" s="3">
-        <v>47876</v>
+        <v>46265</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
-        <v>180</v>
+        <v>290</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>181</v>
+        <v>291</v>
       </c>
       <c r="C4" s="3">
-        <v>47815</v>
+        <v>46265</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="1" t="s">
-        <v>182</v>
+        <v>435</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>183</v>
+        <v>436</v>
       </c>
       <c r="C5" s="3">
-        <v>47780</v>
+        <v>46301</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="1" t="s">
-        <v>184</v>
+        <v>308</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>185</v>
+        <v>309</v>
       </c>
       <c r="C6" s="3">
-        <v>48697</v>
+        <v>46348</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="1" t="s">
-        <v>186</v>
+        <v>443</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>187</v>
+        <v>444</v>
       </c>
       <c r="C7" s="3">
-        <v>49309</v>
+        <v>46436</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="1" t="s">
-        <v>89</v>
+        <v>437</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>189</v>
+        <v>438</v>
       </c>
       <c r="C8" s="3">
-        <v>48915</v>
+        <v>46445</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="1" t="s">
-        <v>190</v>
+        <v>269</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>191</v>
+        <v>270</v>
       </c>
       <c r="C9" s="3">
-        <v>46926</v>
+        <v>46514</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="1" t="s">
-        <v>192</v>
+        <v>439</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>193</v>
+        <v>440</v>
       </c>
       <c r="C10" s="3">
-        <v>49399</v>
+        <v>46527</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="1" t="s">
-        <v>194</v>
+        <v>286</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>195</v>
+        <v>287</v>
       </c>
       <c r="C11" s="3">
-        <v>47822</v>
+        <v>46534</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="1" t="s">
-        <v>196</v>
+        <v>445</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>197</v>
+        <v>446</v>
       </c>
       <c r="C12" s="3">
-        <v>49842</v>
+        <v>46574</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="1" t="s">
-        <v>198</v>
+        <v>298</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>199</v>
+        <v>299</v>
       </c>
       <c r="C13" s="3">
-        <v>48101</v>
+        <v>46582</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="1" t="s">
-        <v>200</v>
+        <v>271</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>201</v>
+        <v>272</v>
       </c>
       <c r="C14" s="3">
-        <v>49294</v>
+        <v>46590</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="1" t="s">
-        <v>202</v>
+        <v>292</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>203</v>
+        <v>293</v>
       </c>
       <c r="C15" s="3">
-        <v>50358</v>
+        <v>46592</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="1" t="s">
-        <v>204</v>
+        <v>247</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>205</v>
+        <v>248</v>
       </c>
       <c r="C16" s="3">
-        <v>50055</v>
+        <v>46610</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>447</v>
@@ -4205,115 +4223,115 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="1" t="s">
-        <v>206</v>
+        <v>86</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>207</v>
+        <v>315</v>
       </c>
       <c r="C17" s="3">
-        <v>47986</v>
+        <v>46690</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="1" t="s">
-        <v>208</v>
+        <v>306</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>209</v>
+        <v>307</v>
       </c>
       <c r="C18" s="3">
-        <v>48364</v>
+        <v>46720</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="1" t="s">
-        <v>210</v>
+        <v>320</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>211</v>
+        <v>321</v>
       </c>
       <c r="C19" s="3">
-        <v>50313</v>
+        <v>46873</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="1" t="s">
-        <v>212</v>
+        <v>294</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>213</v>
+        <v>295</v>
       </c>
       <c r="C20" s="3">
-        <v>47790</v>
+        <v>46901</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="1" t="s">
-        <v>214</v>
+        <v>284</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>215</v>
+        <v>285</v>
       </c>
       <c r="C21" s="3">
-        <v>48047</v>
+        <v>46907</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="1" t="s">
-        <v>88</v>
+        <v>240</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>217</v>
+        <v>241</v>
       </c>
       <c r="C22" s="3">
-        <v>48727</v>
+        <v>46916</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="1" t="s">
-        <v>218</v>
+        <v>190</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>219</v>
+        <v>191</v>
       </c>
       <c r="C23" s="3">
-        <v>49694</v>
+        <v>46926</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>176</v>
@@ -4324,50 +4342,50 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="1" t="s">
-        <v>220</v>
+        <v>322</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>221</v>
+        <v>323</v>
       </c>
       <c r="C24" s="3">
-        <v>48053</v>
+        <v>46945</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="1" t="s">
-        <v>222</v>
+        <v>310</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>223</v>
+        <v>311</v>
       </c>
       <c r="C25" s="3">
-        <v>49633</v>
+        <v>46970</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="1" t="s">
-        <v>224</v>
+        <v>255</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>225</v>
+        <v>256</v>
       </c>
       <c r="C26" s="3">
-        <v>48740</v>
+        <v>46971</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>447</v>
@@ -4375,13 +4393,13 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="1" t="s">
-        <v>226</v>
+        <v>174</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>227</v>
+        <v>175</v>
       </c>
       <c r="C27" s="3">
-        <v>49653</v>
+        <v>47036</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>176</v>
@@ -4392,115 +4410,115 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="1" t="s">
-        <v>228</v>
+        <v>273</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>229</v>
+        <v>274</v>
       </c>
       <c r="C28" s="3">
-        <v>50503</v>
+        <v>47036</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="1" t="s">
-        <v>230</v>
+        <v>324</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>231</v>
+        <v>325</v>
       </c>
       <c r="C29" s="3">
-        <v>47299</v>
+        <v>47072</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="1" t="s">
-        <v>232</v>
+        <v>288</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>233</v>
+        <v>289</v>
       </c>
       <c r="C30" s="3">
-        <v>48102</v>
+        <v>47095</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="1" t="s">
-        <v>234</v>
+        <v>441</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>235</v>
+        <v>442</v>
       </c>
       <c r="C31" s="3">
-        <v>48852</v>
+        <v>47175</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="1" t="s">
-        <v>236</v>
+        <v>263</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>237</v>
+        <v>264</v>
       </c>
       <c r="C32" s="3">
-        <v>48961</v>
+        <v>47176</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="1" t="s">
-        <v>238</v>
+        <v>275</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="C33" s="3">
-        <v>48503</v>
+        <v>47179</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34" s="1" t="s">
-        <v>240</v>
+        <v>316</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>241</v>
+        <v>317</v>
       </c>
       <c r="C34" s="3">
-        <v>46916</v>
+        <v>47182</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>242</v>
@@ -4511,13 +4529,13 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" s="1" t="s">
-        <v>243</v>
+        <v>259</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>244</v>
+        <v>260</v>
       </c>
       <c r="C35" s="3">
-        <v>47274</v>
+        <v>47187</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>242</v>
@@ -4528,13 +4546,13 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" s="1" t="s">
-        <v>245</v>
+        <v>257</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>246</v>
+        <v>258</v>
       </c>
       <c r="C36" s="3">
-        <v>47537</v>
+        <v>47209</v>
       </c>
       <c r="D36" s="1" t="s">
         <v>242</v>
@@ -4545,30 +4563,30 @@
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="1" t="s">
-        <v>247</v>
+        <v>300</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>248</v>
+        <v>301</v>
       </c>
       <c r="C37" s="3">
-        <v>46610</v>
+        <v>47273</v>
       </c>
       <c r="D37" s="1" t="s">
         <v>242</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="1" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="C38" s="3">
-        <v>47357</v>
+        <v>47274</v>
       </c>
       <c r="D38" s="1" t="s">
         <v>242</v>
@@ -4579,81 +4597,78 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="1" t="s">
-        <v>251</v>
+        <v>230</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>252</v>
+        <v>231</v>
       </c>
       <c r="C39" s="3">
-        <v>47388</v>
+        <v>47299</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="1" t="s">
-        <v>253</v>
+        <v>312</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>254</v>
+        <v>313</v>
       </c>
       <c r="C40" s="3">
-        <v>48165</v>
+        <v>47302</v>
       </c>
       <c r="D40" s="1" t="s">
         <v>242</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="1" t="s">
-        <v>255</v>
+        <v>449</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>256</v>
+        <v>450</v>
       </c>
       <c r="C41" s="3">
-        <v>46971</v>
+        <v>47315</v>
       </c>
       <c r="D41" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="E41" s="1" t="s">
-        <v>447</v>
-      </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="1" t="s">
-        <v>257</v>
+        <v>302</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>258</v>
+        <v>303</v>
       </c>
       <c r="C42" s="3">
-        <v>47209</v>
+        <v>47355</v>
       </c>
       <c r="D42" s="1" t="s">
         <v>242</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="1" t="s">
-        <v>259</v>
+        <v>249</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="C43" s="3">
-        <v>47187</v>
+        <v>47357</v>
       </c>
       <c r="D43" s="1" t="s">
         <v>242</v>
@@ -4664,13 +4679,13 @@
     </row>
     <row r="44" spans="1:5">
       <c r="A44" s="1" t="s">
-        <v>261</v>
+        <v>251</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>262</v>
+        <v>252</v>
       </c>
       <c r="C44" s="3">
-        <v>47614</v>
+        <v>47388</v>
       </c>
       <c r="D44" s="1" t="s">
         <v>242</v>
@@ -4681,13 +4696,13 @@
     </row>
     <row r="45" spans="1:5">
       <c r="A45" s="1" t="s">
-        <v>263</v>
+        <v>433</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>264</v>
+        <v>434</v>
       </c>
       <c r="C45" s="3">
-        <v>47176</v>
+        <v>47430</v>
       </c>
       <c r="D45" s="1" t="s">
         <v>242</v>
@@ -4715,30 +4730,30 @@
     </row>
     <row r="47" spans="1:5">
       <c r="A47" s="1" t="s">
-        <v>267</v>
+        <v>245</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>268</v>
+        <v>246</v>
       </c>
       <c r="C47" s="3">
-        <v>48131</v>
+        <v>47537</v>
       </c>
       <c r="D47" s="1" t="s">
         <v>242</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" s="1" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>270</v>
+        <v>277</v>
       </c>
       <c r="C48" s="3">
-        <v>46514</v>
+        <v>47587</v>
       </c>
       <c r="D48" s="1" t="s">
         <v>242</v>
@@ -4749,13 +4764,13 @@
     </row>
     <row r="49" spans="1:5">
       <c r="A49" s="1" t="s">
-        <v>271</v>
+        <v>304</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>272</v>
+        <v>305</v>
       </c>
       <c r="C49" s="3">
-        <v>46590</v>
+        <v>47603</v>
       </c>
       <c r="D49" s="1" t="s">
         <v>242</v>
@@ -4766,13 +4781,13 @@
     </row>
     <row r="50" spans="1:5">
       <c r="A50" s="1" t="s">
-        <v>273</v>
+        <v>261</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>274</v>
+        <v>262</v>
       </c>
       <c r="C50" s="3">
-        <v>47036</v>
+        <v>47614</v>
       </c>
       <c r="D50" s="1" t="s">
         <v>242</v>
@@ -4783,13 +4798,13 @@
     </row>
     <row r="51" spans="1:5">
       <c r="A51" s="1" t="s">
-        <v>275</v>
+        <v>318</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>231</v>
+        <v>319</v>
       </c>
       <c r="C51" s="3">
-        <v>47179</v>
+        <v>47632</v>
       </c>
       <c r="D51" s="1" t="s">
         <v>242</v>
@@ -4800,33 +4815,33 @@
     </row>
     <row r="52" spans="1:5">
       <c r="A52" s="1" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C52" s="3">
-        <v>47587</v>
+        <v>47686</v>
       </c>
       <c r="D52" s="1" t="s">
         <v>242</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="53" spans="1:5">
       <c r="A53" s="1" t="s">
-        <v>278</v>
+        <v>182</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>279</v>
+        <v>183</v>
       </c>
       <c r="C53" s="3">
-        <v>47686</v>
+        <v>47780</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E53" s="1" t="s">
         <v>447</v>
@@ -4834,81 +4849,81 @@
     </row>
     <row r="54" spans="1:5">
       <c r="A54" s="1" t="s">
-        <v>280</v>
+        <v>212</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>281</v>
+        <v>213</v>
       </c>
       <c r="C54" s="3">
-        <v>46265</v>
+        <v>47790</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55" s="1" t="s">
-        <v>282</v>
+        <v>180</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>283</v>
+        <v>181</v>
       </c>
       <c r="C55" s="3">
-        <v>46256</v>
+        <v>47815</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="56" spans="1:5">
       <c r="A56" s="1" t="s">
-        <v>284</v>
+        <v>194</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>285</v>
+        <v>195</v>
       </c>
       <c r="C56" s="3">
-        <v>46907</v>
+        <v>47822</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="57" spans="1:5">
       <c r="A57" s="1" t="s">
-        <v>286</v>
+        <v>178</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>287</v>
+        <v>179</v>
       </c>
       <c r="C57" s="3">
-        <v>46534</v>
+        <v>47876</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="58" spans="1:5">
       <c r="A58" s="1" t="s">
-        <v>288</v>
+        <v>87</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>289</v>
+        <v>297</v>
       </c>
       <c r="C58" s="3">
-        <v>47095</v>
+        <v>47896</v>
       </c>
       <c r="D58" s="1" t="s">
         <v>242</v>
@@ -4919,203 +4934,203 @@
     </row>
     <row r="59" spans="1:5">
       <c r="A59" s="1" t="s">
-        <v>290</v>
+        <v>206</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>291</v>
+        <v>207</v>
       </c>
       <c r="C59" s="3">
-        <v>46265</v>
+        <v>47986</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="60" spans="1:5">
       <c r="A60" s="1" t="s">
-        <v>292</v>
+        <v>214</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>293</v>
+        <v>215</v>
       </c>
       <c r="C60" s="3">
-        <v>46592</v>
+        <v>48047</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="61" spans="1:5">
       <c r="A61" s="1" t="s">
-        <v>294</v>
+        <v>220</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>295</v>
+        <v>221</v>
       </c>
       <c r="C61" s="3">
-        <v>46901</v>
+        <v>48053</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="62" spans="1:5">
       <c r="A62" s="1" t="s">
-        <v>87</v>
+        <v>198</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>297</v>
+        <v>199</v>
       </c>
       <c r="C62" s="3">
-        <v>47896</v>
+        <v>48101</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="63" spans="1:5">
       <c r="A63" s="1" t="s">
-        <v>298</v>
+        <v>232</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>299</v>
+        <v>233</v>
       </c>
       <c r="C63" s="3">
-        <v>46582</v>
+        <v>48102</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="64" spans="1:5">
       <c r="A64" s="1" t="s">
-        <v>300</v>
+        <v>267</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>301</v>
+        <v>268</v>
       </c>
       <c r="C64" s="3">
-        <v>47273</v>
+        <v>48131</v>
       </c>
       <c r="D64" s="1" t="s">
         <v>242</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="65" spans="1:5">
       <c r="A65" s="1" t="s">
-        <v>302</v>
+        <v>253</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>303</v>
+        <v>254</v>
       </c>
       <c r="C65" s="3">
-        <v>47355</v>
+        <v>48165</v>
       </c>
       <c r="D65" s="1" t="s">
         <v>242</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="66" spans="1:5">
       <c r="A66" s="1" t="s">
-        <v>304</v>
+        <v>208</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>305</v>
+        <v>209</v>
       </c>
       <c r="C66" s="3">
-        <v>47603</v>
+        <v>48364</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="67" spans="1:5">
       <c r="A67" s="1" t="s">
-        <v>306</v>
+        <v>238</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>307</v>
+        <v>239</v>
       </c>
       <c r="C67" s="3">
-        <v>46720</v>
+        <v>48503</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="68" spans="1:5">
       <c r="A68" s="1" t="s">
-        <v>308</v>
+        <v>184</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>309</v>
+        <v>185</v>
       </c>
       <c r="C68" s="3">
-        <v>46348</v>
+        <v>48697</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="69" spans="1:5">
       <c r="A69" s="1" t="s">
-        <v>310</v>
+        <v>88</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>311</v>
+        <v>217</v>
       </c>
       <c r="C69" s="3">
-        <v>46970</v>
+        <v>48727</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="70" spans="1:5">
       <c r="A70" s="1" t="s">
-        <v>312</v>
+        <v>224</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>313</v>
+        <v>225</v>
       </c>
       <c r="C70" s="3">
-        <v>47302</v>
+        <v>48740</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E70" s="1" t="s">
         <v>447</v>
@@ -5123,223 +5138,271 @@
     </row>
     <row r="71" spans="1:5">
       <c r="A71" s="1" t="s">
-        <v>86</v>
+        <v>234</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>315</v>
+        <v>235</v>
       </c>
       <c r="C71" s="3">
-        <v>46690</v>
+        <v>48852</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="72" spans="1:5">
       <c r="A72" s="1" t="s">
-        <v>316</v>
+        <v>89</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>317</v>
+        <v>189</v>
       </c>
       <c r="C72" s="3">
-        <v>47182</v>
+        <v>48915</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="73" spans="1:5">
       <c r="A73" s="1" t="s">
-        <v>318</v>
+        <v>236</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>319</v>
+        <v>237</v>
       </c>
       <c r="C73" s="3">
-        <v>47632</v>
+        <v>48961</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="74" spans="1:5">
       <c r="A74" s="1" t="s">
-        <v>320</v>
+        <v>451</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>321</v>
+        <v>452</v>
       </c>
       <c r="C74" s="3">
-        <v>46873</v>
+        <v>49153</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="75" spans="1:5">
       <c r="A75" s="1" t="s">
-        <v>322</v>
+        <v>200</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>323</v>
+        <v>201</v>
       </c>
       <c r="C75" s="3">
-        <v>46945</v>
+        <v>49294</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="76" spans="1:5">
       <c r="A76" s="1" t="s">
-        <v>324</v>
+        <v>186</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>325</v>
+        <v>187</v>
       </c>
       <c r="C76" s="3">
-        <v>47072</v>
+        <v>49309</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="77" spans="1:5">
       <c r="A77" s="1" t="s">
-        <v>433</v>
+        <v>192</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>434</v>
+        <v>193</v>
       </c>
       <c r="C77" s="3">
-        <v>47430</v>
+        <v>49399</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="78" spans="1:5">
       <c r="A78" s="1" t="s">
-        <v>435</v>
+        <v>222</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>436</v>
+        <v>223</v>
       </c>
       <c r="C78" s="3">
-        <v>46301</v>
+        <v>49633</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="79" spans="1:5">
       <c r="A79" s="1" t="s">
-        <v>437</v>
+        <v>226</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>438</v>
+        <v>227</v>
       </c>
       <c r="C79" s="3">
-        <v>46445</v>
+        <v>49653</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="80" spans="1:5">
       <c r="A80" s="1" t="s">
-        <v>439</v>
+        <v>218</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>440</v>
+        <v>219</v>
       </c>
       <c r="C80" s="3">
-        <v>46527</v>
+        <v>49694</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="81" spans="1:5">
       <c r="A81" s="1" t="s">
-        <v>441</v>
+        <v>196</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>442</v>
+        <v>197</v>
       </c>
       <c r="C81" s="3">
-        <v>47175</v>
+        <v>49842</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="82" spans="1:5">
       <c r="A82" s="1" t="s">
-        <v>443</v>
+        <v>453</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>444</v>
+        <v>454</v>
       </c>
       <c r="C82" s="3">
-        <v>46436</v>
+        <v>49856</v>
       </c>
       <c r="D82" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="E82" s="1" t="s">
-        <v>448</v>
-      </c>
     </row>
     <row r="83" spans="1:5">
       <c r="A83" s="1" t="s">
-        <v>445</v>
+        <v>204</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>446</v>
+        <v>205</v>
       </c>
       <c r="C83" s="3">
-        <v>46574</v>
+        <v>50055</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5">
+      <c r="A84" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C84" s="3">
+        <v>50313</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="E84" s="1" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5">
+      <c r="A85" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="C85" s="3">
+        <v>50358</v>
+      </c>
+      <c r="D85" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="E85" s="1" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5">
+      <c r="A86" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="C86" s="3">
+        <v>50503</v>
+      </c>
+      <c r="D86" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="E86" s="1" t="s">
+        <v>447</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Instrumentos: re-agregar TMVE8 (se perdió en el rebase con merge=ours)
El commit anterior rebaseó sobre los flujos de ONs de Ignacio y merge=ours
descartó la versión con TMVE8. Se vuelve a agregar el dual TAMAR/Dólar Linked
sobre la base actual, preservando los datos de ONs/Flujos.
</commit_message>
<xml_diff>
--- a/Instrumentos.xlsx
+++ b/Instrumentos.xlsx
@@ -51858,7 +51858,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEF3529B-9FFE-49C8-A90D-80E2711BFB43}">
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="6" width="16.83203125" customWidth="1"/>
@@ -52352,6 +52352,118 @@
         <v>0.03</v>
       </c>
     </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Fecha Emisión</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Fecha Vencimineto</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>TAMAR aplicable</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Margen</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>TMVE8</t>
+        </is>
+      </c>
+      <c r="B36" s="1" t="inlineStr">
+        <is>
+          <t>TAMAR</t>
+        </is>
+      </c>
+      <c r="C36" s="3">
+        <v>46234</v>
+      </c>
+      <c r="D36" s="3">
+        <v>46783</v>
+      </c>
+      <c r="E36" s="1">
+        <v>10</v>
+      </c>
+      <c r="F36" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Fecha Emisión</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Fecha Vencimineto</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>USD aplicable</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Margen</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>TMVE8</t>
+        </is>
+      </c>
+      <c r="B38" s="1" t="inlineStr">
+        <is>
+          <t>Linked</t>
+        </is>
+      </c>
+      <c r="C38" s="3">
+        <v>46234</v>
+      </c>
+      <c r="D38" s="3">
+        <v>46783</v>
+      </c>
+      <c r="E38" s="1">
+        <v>1499.84</v>
+      </c>
+      <c r="F38" s="4">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Sumar 3 ONs más: ICC6D, NPCED y OZC8D
Aparecieron al reconsultar el filtro de liquidez con la rueda ya avanzada: a la
mañana no llegaban a los 100.000 nominales de volumen promedio y sobre el cierre
sí. El chequeo semanal conviene correrlo con la rueda avanzada.

  ICC6D  B. ICBC 2027             ley local   vol 268.000
  NPCED  Central Puerto Jul-2029  ley local   vol 167.114
  OZC8D  EDEMSA 2033              ley NY      vol 112.200

NPCED lleva el mes en el nombre porque ya existe NPCCD "Central Puerto 2029"
(vence el 25-08-2029).

Divisa de pago: CCL en OZC8D por ser ley NY; las dos de ley local quedan vacías
hasta scrapear el domicilio_pago. Quedan en ⚡ hasta cargar el cronograma.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Instrumentos.xlsx
+++ b/Instrumentos.xlsx
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2927" uniqueCount="455">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2937" uniqueCount="461">
   <si>
     <t>Ticker</t>
   </si>
@@ -1417,6 +1417,24 @@
   <si>
     <t>GEMSA - CTR 2036</t>
   </si>
+  <si>
+    <t>ICC6D</t>
+  </si>
+  <si>
+    <t>B. ICBC 2027</t>
+  </si>
+  <si>
+    <t>NPCED</t>
+  </si>
+  <si>
+    <t>Central Puerto Jul-2029</t>
+  </si>
+  <si>
+    <t>OZC8D</t>
+  </si>
+  <si>
+    <t>EDEMSA 2033</t>
+  </si>
 </sst>
 </file>
 
@@ -3940,7 +3958,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E86"/>
+  <dimension ref="A1:E89"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10"/>
@@ -4121,30 +4139,27 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="1" t="s">
-        <v>286</v>
+        <v>455</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>287</v>
+        <v>456</v>
       </c>
       <c r="C11" s="3">
-        <v>46534</v>
+        <v>46529</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="E11" s="1" t="s">
-        <v>448</v>
-      </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="1" t="s">
-        <v>445</v>
+        <v>286</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>446</v>
+        <v>287</v>
       </c>
       <c r="C12" s="3">
-        <v>46574</v>
+        <v>46534</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>242</v>
@@ -4155,13 +4170,13 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="1" t="s">
-        <v>298</v>
+        <v>445</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>299</v>
+        <v>446</v>
       </c>
       <c r="C13" s="3">
-        <v>46582</v>
+        <v>46574</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>242</v>
@@ -4172,13 +4187,13 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="1" t="s">
-        <v>271</v>
+        <v>298</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>272</v>
+        <v>299</v>
       </c>
       <c r="C14" s="3">
-        <v>46590</v>
+        <v>46582</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>242</v>
@@ -4189,13 +4204,13 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="1" t="s">
-        <v>292</v>
+        <v>271</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>293</v>
+        <v>272</v>
       </c>
       <c r="C15" s="3">
-        <v>46592</v>
+        <v>46590</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>242</v>
@@ -4206,47 +4221,47 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="1" t="s">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>248</v>
+        <v>293</v>
       </c>
       <c r="C16" s="3">
-        <v>46610</v>
+        <v>46592</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>242</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="1" t="s">
-        <v>86</v>
+        <v>247</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>315</v>
+        <v>248</v>
       </c>
       <c r="C17" s="3">
-        <v>46690</v>
+        <v>46610</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>242</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="1" t="s">
-        <v>306</v>
+        <v>86</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="C18" s="3">
-        <v>46720</v>
+        <v>46690</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>242</v>
@@ -4257,13 +4272,13 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="1" t="s">
-        <v>320</v>
+        <v>306</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>321</v>
+        <v>307</v>
       </c>
       <c r="C19" s="3">
-        <v>46873</v>
+        <v>46720</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>242</v>
@@ -4274,13 +4289,13 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="1" t="s">
-        <v>294</v>
+        <v>320</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>295</v>
+        <v>321</v>
       </c>
       <c r="C20" s="3">
-        <v>46901</v>
+        <v>46873</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>242</v>
@@ -4291,13 +4306,13 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="1" t="s">
-        <v>284</v>
+        <v>294</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>285</v>
+        <v>295</v>
       </c>
       <c r="C21" s="3">
-        <v>46907</v>
+        <v>46901</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>242</v>
@@ -4308,13 +4323,13 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="1" t="s">
-        <v>240</v>
+        <v>284</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>241</v>
+        <v>285</v>
       </c>
       <c r="C22" s="3">
-        <v>46916</v>
+        <v>46907</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>242</v>
@@ -4325,47 +4340,47 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="1" t="s">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>191</v>
+        <v>241</v>
       </c>
       <c r="C23" s="3">
-        <v>46926</v>
+        <v>46916</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="1" t="s">
-        <v>322</v>
+        <v>190</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>323</v>
+        <v>191</v>
       </c>
       <c r="C24" s="3">
-        <v>46945</v>
+        <v>46926</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="1" t="s">
-        <v>310</v>
+        <v>322</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>311</v>
+        <v>323</v>
       </c>
       <c r="C25" s="3">
-        <v>46970</v>
+        <v>46945</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>242</v>
@@ -4376,33 +4391,33 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="1" t="s">
-        <v>255</v>
+        <v>310</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>256</v>
+        <v>311</v>
       </c>
       <c r="C26" s="3">
-        <v>46971</v>
+        <v>46970</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>242</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="1" t="s">
-        <v>174</v>
+        <v>255</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>175</v>
+        <v>256</v>
       </c>
       <c r="C27" s="3">
-        <v>47036</v>
+        <v>46971</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>447</v>
@@ -4410,30 +4425,30 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" s="1" t="s">
-        <v>273</v>
+        <v>174</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>274</v>
+        <v>175</v>
       </c>
       <c r="C28" s="3">
         <v>47036</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" s="1" t="s">
-        <v>324</v>
+        <v>273</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>325</v>
+        <v>274</v>
       </c>
       <c r="C29" s="3">
-        <v>47072</v>
+        <v>47036</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>242</v>
@@ -4444,13 +4459,13 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="1" t="s">
-        <v>288</v>
+        <v>324</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>289</v>
+        <v>325</v>
       </c>
       <c r="C30" s="3">
-        <v>47095</v>
+        <v>47072</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>242</v>
@@ -4461,13 +4476,13 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" s="1" t="s">
-        <v>441</v>
+        <v>288</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>442</v>
+        <v>289</v>
       </c>
       <c r="C31" s="3">
-        <v>47175</v>
+        <v>47095</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>242</v>
@@ -4478,13 +4493,13 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" s="1" t="s">
-        <v>263</v>
+        <v>441</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>264</v>
+        <v>442</v>
       </c>
       <c r="C32" s="3">
-        <v>47176</v>
+        <v>47175</v>
       </c>
       <c r="D32" s="1" t="s">
         <v>242</v>
@@ -4495,13 +4510,13 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" s="1" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>231</v>
+        <v>264</v>
       </c>
       <c r="C33" s="3">
-        <v>47179</v>
+        <v>47176</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>242</v>
@@ -4512,13 +4527,13 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" s="1" t="s">
-        <v>316</v>
+        <v>275</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>317</v>
+        <v>231</v>
       </c>
       <c r="C34" s="3">
-        <v>47182</v>
+        <v>47179</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>242</v>
@@ -4529,13 +4544,13 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" s="1" t="s">
-        <v>259</v>
+        <v>316</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>260</v>
+        <v>317</v>
       </c>
       <c r="C35" s="3">
-        <v>47187</v>
+        <v>47182</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>242</v>
@@ -4546,13 +4561,13 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" s="1" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C36" s="3">
-        <v>47209</v>
+        <v>47187</v>
       </c>
       <c r="D36" s="1" t="s">
         <v>242</v>
@@ -4563,13 +4578,13 @@
     </row>
     <row r="37" spans="1:5">
       <c r="A37" s="1" t="s">
-        <v>300</v>
+        <v>257</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>301</v>
+        <v>258</v>
       </c>
       <c r="C37" s="3">
-        <v>47273</v>
+        <v>47209</v>
       </c>
       <c r="D37" s="1" t="s">
         <v>242</v>
@@ -4580,13 +4595,13 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" s="1" t="s">
-        <v>243</v>
+        <v>300</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>244</v>
+        <v>301</v>
       </c>
       <c r="C38" s="3">
-        <v>47274</v>
+        <v>47273</v>
       </c>
       <c r="D38" s="1" t="s">
         <v>242</v>
@@ -4597,33 +4612,33 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="1" t="s">
-        <v>230</v>
+        <v>243</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>231</v>
+        <v>244</v>
       </c>
       <c r="C39" s="3">
-        <v>47299</v>
+        <v>47274</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" s="1" t="s">
-        <v>312</v>
+        <v>230</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>313</v>
+        <v>231</v>
       </c>
       <c r="C40" s="3">
-        <v>47302</v>
+        <v>47299</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E40" s="1" t="s">
         <v>447</v>
@@ -4631,81 +4646,78 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" s="1" t="s">
-        <v>449</v>
+        <v>312</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>450</v>
+        <v>313</v>
       </c>
       <c r="C41" s="3">
-        <v>47315</v>
+        <v>47302</v>
       </c>
       <c r="D41" s="1" t="s">
         <v>242</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="1" t="s">
-        <v>302</v>
+        <v>449</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>303</v>
+        <v>450</v>
       </c>
       <c r="C42" s="3">
-        <v>47355</v>
+        <v>47315</v>
       </c>
       <c r="D42" s="1" t="s">
         <v>242</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43" s="1" t="s">
-        <v>249</v>
+        <v>457</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>250</v>
+        <v>458</v>
       </c>
       <c r="C43" s="3">
-        <v>47357</v>
+        <v>47326</v>
       </c>
       <c r="D43" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="E43" s="1" t="s">
-        <v>448</v>
-      </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" s="1" t="s">
-        <v>251</v>
+        <v>302</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>252</v>
+        <v>303</v>
       </c>
       <c r="C44" s="3">
-        <v>47388</v>
+        <v>47355</v>
       </c>
       <c r="D44" s="1" t="s">
         <v>242</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="45" spans="1:5">
       <c r="A45" s="1" t="s">
-        <v>433</v>
+        <v>249</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>434</v>
+        <v>250</v>
       </c>
       <c r="C45" s="3">
-        <v>47430</v>
+        <v>47357</v>
       </c>
       <c r="D45" s="1" t="s">
         <v>242</v>
@@ -4716,13 +4728,13 @@
     </row>
     <row r="46" spans="1:5">
       <c r="A46" s="1" t="s">
-        <v>265</v>
+        <v>251</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>266</v>
+        <v>252</v>
       </c>
       <c r="C46" s="3">
-        <v>47510</v>
+        <v>47388</v>
       </c>
       <c r="D46" s="1" t="s">
         <v>242</v>
@@ -4733,13 +4745,13 @@
     </row>
     <row r="47" spans="1:5">
       <c r="A47" s="1" t="s">
-        <v>245</v>
+        <v>433</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>246</v>
+        <v>434</v>
       </c>
       <c r="C47" s="3">
-        <v>47537</v>
+        <v>47430</v>
       </c>
       <c r="D47" s="1" t="s">
         <v>242</v>
@@ -4750,13 +4762,13 @@
     </row>
     <row r="48" spans="1:5">
       <c r="A48" s="1" t="s">
-        <v>276</v>
+        <v>265</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>277</v>
+        <v>266</v>
       </c>
       <c r="C48" s="3">
-        <v>47587</v>
+        <v>47510</v>
       </c>
       <c r="D48" s="1" t="s">
         <v>242</v>
@@ -4767,13 +4779,13 @@
     </row>
     <row r="49" spans="1:5">
       <c r="A49" s="1" t="s">
-        <v>304</v>
+        <v>245</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>305</v>
+        <v>246</v>
       </c>
       <c r="C49" s="3">
-        <v>47603</v>
+        <v>47537</v>
       </c>
       <c r="D49" s="1" t="s">
         <v>242</v>
@@ -4784,13 +4796,13 @@
     </row>
     <row r="50" spans="1:5">
       <c r="A50" s="1" t="s">
-        <v>261</v>
+        <v>276</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>262</v>
+        <v>277</v>
       </c>
       <c r="C50" s="3">
-        <v>47614</v>
+        <v>47587</v>
       </c>
       <c r="D50" s="1" t="s">
         <v>242</v>
@@ -4801,13 +4813,13 @@
     </row>
     <row r="51" spans="1:5">
       <c r="A51" s="1" t="s">
-        <v>318</v>
+        <v>304</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>319</v>
+        <v>305</v>
       </c>
       <c r="C51" s="3">
-        <v>47632</v>
+        <v>47603</v>
       </c>
       <c r="D51" s="1" t="s">
         <v>242</v>
@@ -4818,50 +4830,50 @@
     </row>
     <row r="52" spans="1:5">
       <c r="A52" s="1" t="s">
-        <v>278</v>
+        <v>261</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>279</v>
+        <v>262</v>
       </c>
       <c r="C52" s="3">
-        <v>47686</v>
+        <v>47614</v>
       </c>
       <c r="D52" s="1" t="s">
         <v>242</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="53" spans="1:5">
       <c r="A53" s="1" t="s">
-        <v>182</v>
+        <v>318</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>183</v>
+        <v>319</v>
       </c>
       <c r="C53" s="3">
-        <v>47780</v>
+        <v>47632</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54" s="1" t="s">
-        <v>212</v>
+        <v>278</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>213</v>
+        <v>279</v>
       </c>
       <c r="C54" s="3">
-        <v>47790</v>
+        <v>47686</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>447</v>
@@ -4869,13 +4881,13 @@
     </row>
     <row r="55" spans="1:5">
       <c r="A55" s="1" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C55" s="3">
-        <v>47815</v>
+        <v>47780</v>
       </c>
       <c r="D55" s="1" t="s">
         <v>176</v>
@@ -4886,13 +4898,13 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" s="1" t="s">
-        <v>194</v>
+        <v>212</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>195</v>
+        <v>213</v>
       </c>
       <c r="C56" s="3">
-        <v>47822</v>
+        <v>47790</v>
       </c>
       <c r="D56" s="1" t="s">
         <v>176</v>
@@ -4903,13 +4915,13 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" s="1" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C57" s="3">
-        <v>47876</v>
+        <v>47815</v>
       </c>
       <c r="D57" s="1" t="s">
         <v>176</v>
@@ -4920,30 +4932,30 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" s="1" t="s">
-        <v>87</v>
+        <v>194</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>297</v>
+        <v>195</v>
       </c>
       <c r="C58" s="3">
-        <v>47896</v>
+        <v>47822</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="59" spans="1:5">
       <c r="A59" s="1" t="s">
-        <v>206</v>
+        <v>178</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>207</v>
+        <v>179</v>
       </c>
       <c r="C59" s="3">
-        <v>47986</v>
+        <v>47876</v>
       </c>
       <c r="D59" s="1" t="s">
         <v>176</v>
@@ -4954,30 +4966,30 @@
     </row>
     <row r="60" spans="1:5">
       <c r="A60" s="1" t="s">
-        <v>214</v>
+        <v>87</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>215</v>
+        <v>297</v>
       </c>
       <c r="C60" s="3">
-        <v>48047</v>
+        <v>47896</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="61" spans="1:5">
       <c r="A61" s="1" t="s">
-        <v>220</v>
+        <v>206</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>221</v>
+        <v>207</v>
       </c>
       <c r="C61" s="3">
-        <v>48053</v>
+        <v>47986</v>
       </c>
       <c r="D61" s="1" t="s">
         <v>176</v>
@@ -4988,13 +5000,13 @@
     </row>
     <row r="62" spans="1:5">
       <c r="A62" s="1" t="s">
-        <v>198</v>
+        <v>214</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>199</v>
+        <v>215</v>
       </c>
       <c r="C62" s="3">
-        <v>48101</v>
+        <v>48047</v>
       </c>
       <c r="D62" s="1" t="s">
         <v>176</v>
@@ -5005,13 +5017,13 @@
     </row>
     <row r="63" spans="1:5">
       <c r="A63" s="1" t="s">
-        <v>232</v>
+        <v>220</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>233</v>
+        <v>221</v>
       </c>
       <c r="C63" s="3">
-        <v>48102</v>
+        <v>48053</v>
       </c>
       <c r="D63" s="1" t="s">
         <v>176</v>
@@ -5022,16 +5034,16 @@
     </row>
     <row r="64" spans="1:5">
       <c r="A64" s="1" t="s">
-        <v>267</v>
+        <v>198</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>268</v>
+        <v>199</v>
       </c>
       <c r="C64" s="3">
-        <v>48131</v>
+        <v>48101</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E64" s="1" t="s">
         <v>447</v>
@@ -5039,33 +5051,33 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" s="1" t="s">
-        <v>253</v>
+        <v>232</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>254</v>
+        <v>233</v>
       </c>
       <c r="C65" s="3">
-        <v>48165</v>
+        <v>48102</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="66" spans="1:5">
       <c r="A66" s="1" t="s">
-        <v>208</v>
+        <v>267</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>209</v>
+        <v>268</v>
       </c>
       <c r="C66" s="3">
-        <v>48364</v>
+        <v>48131</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E66" s="1" t="s">
         <v>447</v>
@@ -5073,30 +5085,30 @@
     </row>
     <row r="67" spans="1:5">
       <c r="A67" s="1" t="s">
-        <v>238</v>
+        <v>253</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>239</v>
+        <v>254</v>
       </c>
       <c r="C67" s="3">
-        <v>48503</v>
+        <v>48165</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="68" spans="1:5">
       <c r="A68" s="1" t="s">
-        <v>184</v>
+        <v>208</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="C68" s="3">
-        <v>48697</v>
+        <v>48364</v>
       </c>
       <c r="D68" s="1" t="s">
         <v>176</v>
@@ -5107,13 +5119,13 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" s="1" t="s">
-        <v>88</v>
+        <v>238</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="C69" s="3">
-        <v>48727</v>
+        <v>48503</v>
       </c>
       <c r="D69" s="1" t="s">
         <v>176</v>
@@ -5124,13 +5136,13 @@
     </row>
     <row r="70" spans="1:5">
       <c r="A70" s="1" t="s">
-        <v>224</v>
+        <v>184</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>225</v>
+        <v>185</v>
       </c>
       <c r="C70" s="3">
-        <v>48740</v>
+        <v>48697</v>
       </c>
       <c r="D70" s="1" t="s">
         <v>176</v>
@@ -5141,13 +5153,13 @@
     </row>
     <row r="71" spans="1:5">
       <c r="A71" s="1" t="s">
-        <v>234</v>
+        <v>88</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>235</v>
+        <v>217</v>
       </c>
       <c r="C71" s="3">
-        <v>48852</v>
+        <v>48727</v>
       </c>
       <c r="D71" s="1" t="s">
         <v>176</v>
@@ -5158,13 +5170,13 @@
     </row>
     <row r="72" spans="1:5">
       <c r="A72" s="1" t="s">
-        <v>89</v>
+        <v>224</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>189</v>
+        <v>225</v>
       </c>
       <c r="C72" s="3">
-        <v>48915</v>
+        <v>48740</v>
       </c>
       <c r="D72" s="1" t="s">
         <v>176</v>
@@ -5175,13 +5187,13 @@
     </row>
     <row r="73" spans="1:5">
       <c r="A73" s="1" t="s">
-        <v>236</v>
+        <v>459</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>237</v>
+        <v>460</v>
       </c>
       <c r="C73" s="3">
-        <v>48961</v>
+        <v>48741</v>
       </c>
       <c r="D73" s="1" t="s">
         <v>176</v>
@@ -5192,13 +5204,13 @@
     </row>
     <row r="74" spans="1:5">
       <c r="A74" s="1" t="s">
-        <v>451</v>
+        <v>234</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>452</v>
+        <v>235</v>
       </c>
       <c r="C74" s="3">
-        <v>49153</v>
+        <v>48852</v>
       </c>
       <c r="D74" s="1" t="s">
         <v>176</v>
@@ -5209,13 +5221,13 @@
     </row>
     <row r="75" spans="1:5">
       <c r="A75" s="1" t="s">
-        <v>200</v>
+        <v>89</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>201</v>
+        <v>189</v>
       </c>
       <c r="C75" s="3">
-        <v>49294</v>
+        <v>48915</v>
       </c>
       <c r="D75" s="1" t="s">
         <v>176</v>
@@ -5226,13 +5238,13 @@
     </row>
     <row r="76" spans="1:5">
       <c r="A76" s="1" t="s">
-        <v>186</v>
+        <v>236</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>187</v>
+        <v>237</v>
       </c>
       <c r="C76" s="3">
-        <v>49309</v>
+        <v>48961</v>
       </c>
       <c r="D76" s="1" t="s">
         <v>176</v>
@@ -5243,13 +5255,13 @@
     </row>
     <row r="77" spans="1:5">
       <c r="A77" s="1" t="s">
-        <v>192</v>
+        <v>451</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>193</v>
+        <v>452</v>
       </c>
       <c r="C77" s="3">
-        <v>49399</v>
+        <v>49153</v>
       </c>
       <c r="D77" s="1" t="s">
         <v>176</v>
@@ -5260,13 +5272,13 @@
     </row>
     <row r="78" spans="1:5">
       <c r="A78" s="1" t="s">
-        <v>222</v>
+        <v>200</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>223</v>
+        <v>201</v>
       </c>
       <c r="C78" s="3">
-        <v>49633</v>
+        <v>49294</v>
       </c>
       <c r="D78" s="1" t="s">
         <v>176</v>
@@ -5277,13 +5289,13 @@
     </row>
     <row r="79" spans="1:5">
       <c r="A79" s="1" t="s">
-        <v>226</v>
+        <v>186</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>227</v>
+        <v>187</v>
       </c>
       <c r="C79" s="3">
-        <v>49653</v>
+        <v>49309</v>
       </c>
       <c r="D79" s="1" t="s">
         <v>176</v>
@@ -5294,13 +5306,13 @@
     </row>
     <row r="80" spans="1:5">
       <c r="A80" s="1" t="s">
-        <v>218</v>
+        <v>192</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>219</v>
+        <v>193</v>
       </c>
       <c r="C80" s="3">
-        <v>49694</v>
+        <v>49399</v>
       </c>
       <c r="D80" s="1" t="s">
         <v>176</v>
@@ -5311,13 +5323,13 @@
     </row>
     <row r="81" spans="1:5">
       <c r="A81" s="1" t="s">
-        <v>196</v>
+        <v>222</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>197</v>
+        <v>223</v>
       </c>
       <c r="C81" s="3">
-        <v>49842</v>
+        <v>49633</v>
       </c>
       <c r="D81" s="1" t="s">
         <v>176</v>
@@ -5328,30 +5340,30 @@
     </row>
     <row r="82" spans="1:5">
       <c r="A82" s="1" t="s">
-        <v>453</v>
+        <v>226</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>454</v>
+        <v>227</v>
       </c>
       <c r="C82" s="3">
-        <v>49856</v>
+        <v>49653</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>242</v>
+        <v>176</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="83" spans="1:5">
       <c r="A83" s="1" t="s">
-        <v>204</v>
+        <v>218</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>205</v>
+        <v>219</v>
       </c>
       <c r="C83" s="3">
-        <v>50055</v>
+        <v>49694</v>
       </c>
       <c r="D83" s="1" t="s">
         <v>176</v>
@@ -5362,13 +5374,13 @@
     </row>
     <row r="84" spans="1:5">
       <c r="A84" s="1" t="s">
-        <v>210</v>
+        <v>196</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>211</v>
+        <v>197</v>
       </c>
       <c r="C84" s="3">
-        <v>50313</v>
+        <v>49842</v>
       </c>
       <c r="D84" s="1" t="s">
         <v>176</v>
@@ -5379,35 +5391,86 @@
     </row>
     <row r="85" spans="1:5">
       <c r="A85" s="1" t="s">
-        <v>202</v>
+        <v>453</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>203</v>
+        <v>454</v>
       </c>
       <c r="C85" s="3">
-        <v>50358</v>
+        <v>49856</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>176</v>
+        <v>242</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="86" spans="1:5">
       <c r="A86" s="1" t="s">
-        <v>228</v>
+        <v>204</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>229</v>
+        <v>205</v>
       </c>
       <c r="C86" s="3">
-        <v>50503</v>
+        <v>50055</v>
       </c>
       <c r="D86" s="1" t="s">
         <v>176</v>
       </c>
       <c r="E86" s="1" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5">
+      <c r="A87" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C87" s="3">
+        <v>50313</v>
+      </c>
+      <c r="D87" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="E87" s="1" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5">
+      <c r="A88" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="C88" s="3">
+        <v>50358</v>
+      </c>
+      <c r="D88" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="E88" s="1" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5">
+      <c r="A89" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="C89" s="3">
+        <v>50503</v>
+      </c>
+      <c r="D89" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="E89" s="1" t="s">
         <v>447</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Instrumentos: reunir el TMVE8 de Fran con las 3 ONs nuevas
El merge con fork/main descartó en silencio el TMVE8: .gitattributes marca
Instrumentos.xlsx con merge=ours, así que git se quedó con nuestra versión sin
avisar. Es la misma pérdida que Fran tuvo que revertir en ac6c5a5.

Se reconstruyó la unión partiendo del archivo de Fran (que trae TMVE8 en Duales
con sus dos patas, TAMAR y Linked) y re-aplicando encima ICC6D, NPCED y OZC8D
con sus cash flows y divisa de pago, que sólo tocan las hojas ONs y Flujos.

Verificado: 1429 fórmulas, 13 hojas, TMVE8 con 2 patas, 88 ONs y 1611 flujos
(las 6 ONs nuevas suman 66).

Nota para la próxima: al mergear upstream hay que revisar a mano si el otro lado
tocó Instrumentos.xlsx o historicos.xlsx; merge=ours no marca conflicto.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Instrumentos.xlsx
+++ b/Instrumentos.xlsx
@@ -52407,7 +52407,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEF3529B-9FFE-49C8-A90D-80E2711BFB43}">
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="6" width="16.83203125" customWidth="1"/>
@@ -52901,6 +52901,118 @@
         <v>0.03</v>
       </c>
     </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Fecha Emisión</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Fecha Vencimineto</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>TAMAR aplicable</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Margen</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>TMVE8</t>
+        </is>
+      </c>
+      <c r="B36" s="1" t="inlineStr">
+        <is>
+          <t>TAMAR</t>
+        </is>
+      </c>
+      <c r="C36" s="3">
+        <v>46234</v>
+      </c>
+      <c r="D36" s="3">
+        <v>46783</v>
+      </c>
+      <c r="E36" s="1">
+        <v>10</v>
+      </c>
+      <c r="F36" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Fecha Emisión</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Fecha Vencimineto</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>USD aplicable</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Margen</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>TMVE8</t>
+        </is>
+      </c>
+      <c r="B38" s="1" t="inlineStr">
+        <is>
+          <t>Linked</t>
+        </is>
+      </c>
+      <c r="C38" s="3">
+        <v>46234</v>
+      </c>
+      <c r="D38" s="3">
+        <v>46783</v>
+      </c>
+      <c r="E38" s="1">
+        <v>1499.84</v>
+      </c>
+      <c r="F38" s="4">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>